<commit_message>
addition of s2 minibus use logic and final notebook pull of all files
</commit_message>
<xml_diff>
--- a/notebooks/outputs/prm_v2/monthly_summary_v2/monthly_summary.xlsx
+++ b/notebooks/outputs/prm_v2/monthly_summary_v2/monthly_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="18">
   <si>
     <t>month</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
   </si>
   <si>
     <t>P100</t>
@@ -422,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -459,7 +462,7 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>99.74221882757304</v>
@@ -480,7 +483,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -488,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -509,7 +512,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -517,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4">
         <v>99.99034003091191</v>
@@ -538,7 +541,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -546,7 +549,7 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <v>99.98941462898274</v>
@@ -567,7 +570,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -575,7 +578,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -596,7 +599,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -604,7 +607,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -625,6 +628,64 @@
         <v>0</v>
       </c>
       <c r="I7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8">
+        <v>99.87974098057354</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>55</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>100</v>
+      </c>
+      <c r="D9">
+        <v>11</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>47</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>